<commit_message>
Fix artifact contents and revision-history ordering
The previous commit staged the renamed documents with git mv, which
captured their pre-edit content: the published SCO, IRP and REG binaries
were the old v1.2, v1.2 and v1.0 documents under the new filenames, so
none of the entity-classification corrections were actually delivered.
Re-stage the edited DOCX sources and their re-exported PDFs.

Order the revision-history tables chronologically. The v1.1 rows had been
appended after v1.2 rather than inserted after 1.0, so SCO, IRP and POL
read 1.0 / 1.2 / 1.1 (/ 1.3) instead of ascending.

Correct the SoA v1.2 version-history cell that stored 1.1 as the float
1.1000000000000001 instead of text.

Exports remain A4 with no blank pages: POL 12pp, SCO 18pp, IRP 6pp.
</commit_message>
<xml_diff>
--- a/3_Statement_of_Applicability/MT-ISMS-SOA-001_v1.2_statement-of-applicability.xlsx
+++ b/3_Statement_of_Applicability/MT-ISMS-SOA-001_v1.2_statement-of-applicability.xlsx
@@ -4506,8 +4506,10 @@
       </c>
     </row>
     <row r="6" spans="2:5" ht="85" x14ac:dyDescent="0.2">
-      <c r="B6" s="27">
-        <v>1.1000000000000001</v>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
       </c>
       <c r="C6" s="25" t="s">
         <v>3</v>

</xml_diff>